<commit_message>
Complete Hoi P'loy July 2026 recon: all 13 checks, findings register, dashboard, TB calibration and Xero export adapters
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0152b3XNebe3DVRjBHQucxCQ
</commit_message>
<xml_diff>
--- a/recon/hoi-ploy/audit_pack_2026-07.xlsx
+++ b/recon/hoi-ploy/audit_pack_2026-07.xlsx
@@ -14,7 +14,7 @@
     <sheet name="COGS reconciliation (investigat" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Pending purchase orders review" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Sale credit notes not restocked" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="tb" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Trial Balance - Cin7 vs Xero" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Stock received vs invoiced" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Transactions vs stock on hand (" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Outstanding quotes review" sheetId="11" state="visible" r:id="rId11"/>
@@ -33,7 +33,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;(#,##0.00);-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,17 +100,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C8CFD4"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00DADACF"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -130,11 +124,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E4C46A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C8CFD4"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,16 +164,14 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -571,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>July 2026  |  generated 2026-07-31T10:48:50  |  cadence: monthly</t>
+          <t>July 2026  |  generated 2026-07-31T10:58:10  |  cadence: monthly</t>
         </is>
       </c>
     </row>
@@ -582,7 +569,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.292</v>
+        <v>0.269</v>
       </c>
     </row>
     <row r="5">
@@ -593,7 +580,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6 / 5 / 0</t>
+          <t>7 / 5 / 0</t>
         </is>
       </c>
     </row>
@@ -794,7 +781,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>tb</t>
+          <t>Trial Balance - Cin7 vs Xero</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -802,17 +789,20 @@
           <t>Both systems</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>NOT_RUN</t>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ACTION</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>9974.290000000001</v>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Not run - engine error: Xero Trial Balance: could not find Debit/Credit header row</t>
+          <t>3 accounts with large Cin7-vs-Xero gaps, 1 small diffs, 1 Cin7 accounts unmatched in Xero (99 tie clean; 32 expected finance/Xero-only)</t>
         </is>
       </c>
     </row>
@@ -936,7 +926,7 @@
           <t>Cin7</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
@@ -982,13 +972,13 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Total exceptions</t>
         </is>
       </c>
-      <c r="D21" s="13" t="n">
-        <v>353</v>
+      <c r="D21" s="12" t="n">
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -1028,46 +1018,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 114</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Each line is a document whose GL posting disagrees with the stock ledger - classic causes: assemblies posted before completion (WIP), in-transit transfers straddling the period end, and purchases with GRNI timing. Open each task in Cin7, confirm which side is right, and re-post/complete.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Task #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Transaction Type</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Stock Amount</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Document Amount</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
@@ -4074,46 +4064,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Status: WATCH   Exceptions: 63</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Follow up or void: quotes left open clutter the pipeline and can be converted twice. Convert to sale, or void with a reason.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Order #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Rep</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Lines</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -5793,41 +5783,41 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Status: WATCH   Exceptions: 35</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Pending orders are unfulfilled demand: pick/pack/invoice them, or void if the customer cancelled. Anything pending across a month-end understates revenue in the period the customer expected.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Order #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Lines</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
@@ -6671,26 +6661,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Status: INFO   Exceptions: 0</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: The stock-on-hand value should tie to the inventory control accounts on the Balance Sheet; Due should tie to AR. Identity failures mean a sale row was edited inconsistently - open the failing invoices in Cin7.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -6963,46 +6953,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 5</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: A negative GP% often means a costing error (wrong unit cost, missing assembly cost) rather than genuine below-cost selling - verify the SKU's cost before repricing. Deep-loss SKUs (&lt;= -20%) first.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Sku</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Cogs</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Gp</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Gp_Pct</t>
         </is>
@@ -7404,41 +7394,41 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Most errors mean Cin7 re-pushed a document already PAID in Xero. If Xero is correct: Cin7 -&gt; Xero Sync History -&gt; set entry to Skipped (bulk-select Failed/Warning works). If the Cin7 change must reach Xero: remove the payment in Xero, re-sync, re-apply the payment.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Cin7 Core Number</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Issue Type</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
@@ -7534,41 +7524,41 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Sections 1/3: document exists in Xero only - usually manual Xero entries or consolidated Cin7 pushes; confirm intent, then create or sync the Cin7 side or accept as Xero-manual. Sections 2/4: Cin7 document never reached Xero - check Xero Sync History and re-sync. Section 5: line-level edits in one system only - open both documents and align.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Document</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Xero</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Cin7</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
@@ -7626,46 +7616,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 5</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: A credited sale should net to zero due. Open each credit note in Cin7, allocate it against its invoice (or refund it), and confirm the pair washes to nil in Xero AR.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Invoice #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Order Date</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Invoice</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
@@ -7844,26 +7834,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Status: WATCH   Exceptions: 0</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Differences come from bundles/kits (assembly cost-out lands in FinishedGoods), consignment/channel locations, and order status timing. A large or growing gap can mean COGS is misstated in one system - trace the by-type and by-location breakdown.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -8050,66 +8040,66 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Status: WATCH   Exceptions: 65</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Work each line: enter the supplier invoice where stock is received but uninvoiced, receive stock where invoiced but not received, and void stale orders that will never be fulfilled.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Po #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Po Date</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Sku</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Ordered</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>To Invoice</t>
         </is>
       </c>
-      <c r="I6" s="16" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>To Receive</t>
         </is>
       </c>
-      <c r="J6" s="16" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>Action Needed</t>
         </is>
@@ -11143,51 +11133,51 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Status: WATCH   Exceptions: 11</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Per SKU, credited units should re-enter stock (Sale/SaleMultiple, Type=In) unless genuinely not returned (damaged/kept). Restock the missing units in Cin7, or record why not (write-off) so inventory and COGS stay true. Service-only credit lines (shipping, fees) are excluded.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Sku</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Cn_Docs</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Qty_Credited</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Qty_Restocked</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Shortfall</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Cn_Value</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Restock Status</t>
         </is>
@@ -11523,34 +11513,3526 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>tb</t>
+          <t>Trial Balance - Cin7 vs Xero</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Not run - engine error: Xero Trial Balance: could not find Debit/Credit header row</t>
+          <t>3 accounts with large Cin7-vs-Xero gaps, 1 small diffs, 1 Cin7 accounts unmatched in Xero (99 tie clean; 32 expected finance/Xero-only)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
-        <is>
-          <t>Status: NOT_RUN   Exceptions: 0</t>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Status: ACTION   Exceptions: 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>How to resolve: This is a difference map, not a tie-out: Xero carries finance activity (bank, VAT, payroll, journals) Cin7 never sees - those are tagged Expected and not flagged. A REVIEW gap means Cin7 posted movement that never landed in Xero (or vice versa): cross-check the account against the Xero sync failures and the sales recon, and fix the sync, not the ledger.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>No exception rows.</t>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Cin7</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Xero</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>449 Product development</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>6505.13</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>1521.13</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>4984</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>REVIEW - large gap (possible sync issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>203 Lamp Holders</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>-55014.77</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-57864.77</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>2850</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>REVIEW - large gap (possible sync issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>448 Delivery - Local COS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>2220.29</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>-2140.29</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>REVIEW - large gap (possible sync issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>507.2 Commission Control Account (Adj.)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>No Xero match (check account mapping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>229 Delivery - National</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>-18116.65</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-18346.65</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Small diff</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>100 Hoi P'loy (PTY) LTD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>358129.67</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>72169.13</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>285960.54</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>108 YOCO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>191648.36</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>-1510.13</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>193158.49</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>102 Payfast</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>185440.75</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>37093.13</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>148347.62</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>559 Supplier Control Account</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>395557.47</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>494659.76</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>-99102.28999999999</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>503 Loan Account: General</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>-1461.14</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>-18303.26</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>16842.12</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>565 VAT Payable</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>-148338.15</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>-133281.92</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>-15056.23</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>507 Customer Control Account</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>4435.39</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>15663.89</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>-11228.5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Expected - finance/non-inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>411 Advertising, marketing and promotions</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>41984.49</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>-41984.49</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>105 FNB Credit Card</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>11071.11</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>-11071.11</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>464 Research and Development</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>4984</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>-4984</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>429 Safety and Security</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>1340.54</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>-1340.54</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>438 Workshop expense</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>919.96</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>-919.96</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>422 Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>750</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>-750</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>456 Bank charges - Snapscan</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>702.3</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>-702.3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>906 Office Expense</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>698.48</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>-698.48</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>445 Bank Charges Forex Payments</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>536.54</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>-536.54</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>499 Realised Currency Gains</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>462.84</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>-462.84</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>412 Bank Charges - Cheque Acc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>-100</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>420 Printing &amp; Stationery</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>95.65000000000001</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>-95.65000000000001</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Xero-only activity (no Cin7 movement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>108.1 Yoco Bank (Adj)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>109 Payflex</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>505 Deposit - Rent</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>509 Supplier Deposits Account (Dear)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>510 Yoco Control Account</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>328 Customs VAT control</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>416 Office Consumables</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>452 Stationery</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>550 VAT Provision</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>566 Customer Credits (Dear)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>-1 Sales</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>225 Gift voucher</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>252 Discount Received</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Dormant in Cin7 - no Xero match (not flagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>564 Rounding</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>524 Packaging Inv</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>306.37</v>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>306.28</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>537 Light bulbs Inv</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>-10651.16</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>-10651.08</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>520 Components Inv</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>-10579.23</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>-10579.19</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>535 Cable Grips Inv</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>17444.42</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>17444.38</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>301 Inventory discrepancy (Dear)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>-3573.17</v>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>-3573.21</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>315 Lamp Holders COGS</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="n">
+        <v>10386.61</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>10386.57</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>319 Fabric Cables COGS</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="n">
+        <v>40746.69</v>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>40746.65</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>501 Inventory</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>4831.18</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>4831.21</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>529 Fabric Cables Inv</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>-31978.23</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>-31978.2</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>532 Lamp Holders Inv</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="n">
+        <v>-19902.13</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>-19902.1</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>313 Ceiling Cups COGS</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="n">
+        <v>22632.28</v>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>22632.25</v>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>312 Ceiling Pendants COGS</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>36187.19</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>36187.21</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>314 Wall Sconces COGS</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="n">
+        <v>42332.06</v>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>42332.08</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>322 Light bulbs COGS</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="n">
+        <v>20498.45</v>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>20498.47</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>500 Raw Materials</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="n">
+        <v>-146.89</v>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>-146.9</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>521 Ceiling Pendants Inv</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>523 Ceiling Cups Inv</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="n">
+        <v>-21658.16</v>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>-21658.17</v>
+      </c>
+      <c r="E61" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>526 HP Hardware Inv</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="n">
+        <v>-7640.08</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>-7640.09</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>531 Accessories Inv</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="n">
+        <v>-457.36</v>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>-457.35</v>
+      </c>
+      <c r="E63" s="9" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>533 Wall Sconces Inv</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="n">
+        <v>-859.25</v>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>-859.26</v>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>538 Product Finishing Inv</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="n">
+        <v>-1262.11</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>-1262.1</v>
+      </c>
+      <c r="E65" s="9" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>309 Product Finishing COGS</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="n">
+        <v>-624.64</v>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>-624.65</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>317 Pendant Lights COGS</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="n">
+        <v>878.62</v>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>878.63</v>
+      </c>
+      <c r="E67" s="9" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>103 Petty Cash</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>502 Loan Account: Other</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>504 Investments</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>507.1 Customer Control Account (Adj)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>508 Inventory (Dear)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>511 Goods Received Not Invoiced</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="n">
+        <v>-91894.27</v>
+      </c>
+      <c r="D73" s="9" t="n">
+        <v>-91894.27</v>
+      </c>
+      <c r="E73" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>512 Goods Invoiced Not Received</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="n">
+        <v>15150</v>
+      </c>
+      <c r="D74" s="9" t="n">
+        <v>15150</v>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>514 Nat &amp; Mae - Packaging Inventory</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>522 Table Lamps Inv</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>525 Pendant Lights Inv</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>527 String Lights Inv</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>530 Wall Lights Inv</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="n">
+        <v>-369.82</v>
+      </c>
+      <c r="D79" s="9" t="n">
+        <v>-369.82</v>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>534 Stationery Inv</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>536 Porky Heffer Collaboration Inv</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>539 Molecules Inv</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>703 2.Fixed Assets - Accum Dep - Equipment</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>708 2.Fixed Assets - Equipment</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>709 3.Fixed Assets - Furniture &amp; Fittings</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>711 Property - 48 Hopkins, Salt River</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>716 Stock in transit</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>300 Cost of Goods Sold (Dear)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="n">
+        <v>5462.82</v>
+      </c>
+      <c r="D88" s="9" t="n">
+        <v>5462.82</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>303 Cost of Sales / Purchases</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>306 Accessories COGS</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="n">
+        <v>6177.98</v>
+      </c>
+      <c r="D90" s="9" t="n">
+        <v>6177.98</v>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>307 Packaging COGS</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="n">
+        <v>9428.16</v>
+      </c>
+      <c r="D91" s="9" t="n">
+        <v>9428.16</v>
+      </c>
+      <c r="E91" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>308 Courier COGS</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>311 Components COGS</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="n">
+        <v>5665.5</v>
+      </c>
+      <c r="D93" s="9" t="n">
+        <v>5665.5</v>
+      </c>
+      <c r="E93" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>316 Table Lamps COGS</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>318 Cable Grips COGS</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="n">
+        <v>5844.69</v>
+      </c>
+      <c r="D95" s="9" t="n">
+        <v>5844.69</v>
+      </c>
+      <c r="E95" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>320 Custom COGS</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="n">
+        <v>948</v>
+      </c>
+      <c r="D96" s="9" t="n">
+        <v>948</v>
+      </c>
+      <c r="E96" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>321 Process COGS</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>323 Molecules COGS</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>324 Wall Lights COGS</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="n">
+        <v>20196.24</v>
+      </c>
+      <c r="D99" s="9" t="n">
+        <v>20196.24</v>
+      </c>
+      <c r="E99" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>325 String Lights COGS</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="n">
+        <v>10835.18</v>
+      </c>
+      <c r="D100" s="9" t="n">
+        <v>10835.18</v>
+      </c>
+      <c r="E100" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>326 Customer Credits Written Off</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>327 Porky Heffer COGS</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>372 HP Hardware COGS</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="n">
+        <v>4775.02</v>
+      </c>
+      <c r="D103" s="9" t="n">
+        <v>4775.02</v>
+      </c>
+      <c r="E103" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>373 Stationery COGS</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="n">
+        <v>98.16</v>
+      </c>
+      <c r="D104" s="9" t="n">
+        <v>98.16</v>
+      </c>
+      <c r="E104" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>374 Popstruckt Furniture COGS</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>433 Bad Debts</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>450 Designer Commission</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>458 Donations</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>469 Customs Duty</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>470 Delivery - International COS</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>471 Delivery - National COS</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>482 Nat &amp; Mae - Marketing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>912 Nat &amp; Mae - Product Costs</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>913 Nat &amp; Mae - Product Dev</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>554 Suspense</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>567 Gift Card Liability (Dear)</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>902 System Rounding</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>200 Sales</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="n">
+        <v>-42878.93</v>
+      </c>
+      <c r="D118" s="9" t="n">
+        <v>-42878.93</v>
+      </c>
+      <c r="E118" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>201 Porky Heffer Collaboration</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>202 Light Bulbs</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="n">
+        <v>-109132.42</v>
+      </c>
+      <c r="D120" s="9" t="n">
+        <v>-109132.42</v>
+      </c>
+      <c r="E120" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>204 Packaging</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>205 Wall Lights</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="n">
+        <v>-112399.58</v>
+      </c>
+      <c r="D122" s="9" t="n">
+        <v>-112399.58</v>
+      </c>
+      <c r="E122" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>206 String Lights</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="n">
+        <v>-30336.55</v>
+      </c>
+      <c r="D123" s="9" t="n">
+        <v>-30336.55</v>
+      </c>
+      <c r="E123" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>207 Other Sales</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>208 Components</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="n">
+        <v>-29300.89</v>
+      </c>
+      <c r="D125" s="9" t="n">
+        <v>-29300.89</v>
+      </c>
+      <c r="E125" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>209 Ceiling Cups</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="n">
+        <v>-50303.57</v>
+      </c>
+      <c r="D126" s="9" t="n">
+        <v>-50303.57</v>
+      </c>
+      <c r="E126" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>210 Accessories</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="n">
+        <v>-18574.89</v>
+      </c>
+      <c r="D127" s="9" t="n">
+        <v>-18574.89</v>
+      </c>
+      <c r="E127" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>211 Fabric Cables</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="n">
+        <v>-121945.23</v>
+      </c>
+      <c r="D128" s="9" t="n">
+        <v>-121945.23</v>
+      </c>
+      <c r="E128" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>212 Table Lamps</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>213 Ceiling Pendants</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="n">
+        <v>-191998.7</v>
+      </c>
+      <c r="D130" s="9" t="n">
+        <v>-191998.7</v>
+      </c>
+      <c r="E130" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>216 Wall Sconces</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="n">
+        <v>-238090.88</v>
+      </c>
+      <c r="D131" s="9" t="n">
+        <v>-238090.88</v>
+      </c>
+      <c r="E131" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>218 Molecules</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="n">
+        <v>-13147.83</v>
+      </c>
+      <c r="D132" s="9" t="n">
+        <v>-13147.83</v>
+      </c>
+      <c r="E132" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>219 Delivery - Local</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="n">
+        <v>-8020.33</v>
+      </c>
+      <c r="D133" s="9" t="n">
+        <v>-8020.33</v>
+      </c>
+      <c r="E133" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>220 Sales (Dear)</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="n">
+        <v>-11747.57</v>
+      </c>
+      <c r="D134" s="9" t="n">
+        <v>-11747.57</v>
+      </c>
+      <c r="E134" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>222 Pendant Lights</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="n">
+        <v>-2582.61</v>
+      </c>
+      <c r="D135" s="9" t="n">
+        <v>-2582.61</v>
+      </c>
+      <c r="E135" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>223 Cable Grips</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="n">
+        <v>-9009.74</v>
+      </c>
+      <c r="D136" s="9" t="n">
+        <v>-9009.74</v>
+      </c>
+      <c r="E136" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>224 Custom</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="n">
+        <v>-5723.6</v>
+      </c>
+      <c r="D137" s="9" t="n">
+        <v>-5723.6</v>
+      </c>
+      <c r="E137" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>226 Product finishing</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="n">
+        <v>-4173.92</v>
+      </c>
+      <c r="D138" s="9" t="n">
+        <v>-4173.92</v>
+      </c>
+      <c r="E138" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>230 Delivery - International</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>272 HP Hardware</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="n">
+        <v>-773.92</v>
+      </c>
+      <c r="D140" s="9" t="n">
+        <v>-773.92</v>
+      </c>
+      <c r="E140" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>273 Stationery</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>274 Popstrukt Furniture</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>OK (tie)</t>
         </is>
       </c>
     </row>
@@ -11595,66 +15077,66 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Status: ACTION   Exceptions: 52</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>How to resolve: Received &gt; invoiced: chase and capture the supplier invoice - until then the value sits in GRNI and creditors are understated. Invoiced &gt; received: confirm the stock is genuinely in transit, or the invoice was over-captured.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Po #</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Invoice #</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Sku</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Received</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Invoiced</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
-      <c r="I6" s="16" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>Po Total</t>
         </is>
       </c>
-      <c r="J6" s="16" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>